<commit_message>
Update AIP retail diesel prices
</commit_message>
<xml_diff>
--- a/data/diesel_weekly_prices.xlsx
+++ b/data/diesel_weekly_prices.xlsx
@@ -1,70 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>month_start</t>
-  </si>
-  <si>
-    <t>week_ending</t>
-  </si>
-  <si>
-    <t>Sydney</t>
-  </si>
-  <si>
-    <t>Canberra</t>
-  </si>
-  <si>
-    <t>Melbourne</t>
-  </si>
-  <si>
-    <t>Brisbane</t>
-  </si>
-  <si>
-    <t>Adelaide</t>
-  </si>
-  <si>
-    <t>Perth</t>
-  </si>
-  <si>
-    <t>Darwin</t>
-  </si>
-  <si>
-    <t>Hobart</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -83,14 +50,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -378,1707 +412,1731 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J53"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="1">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month_start</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>week_ending</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Canberra</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Adelaide</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Perth</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Darwin</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Hobart</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
         <v>45870</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="1" t="n">
         <v>45900</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>180.2</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>193.4</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>185.3</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>186.5</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>179.1</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="n">
         <v>179.7</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="n">
         <v>187.1</v>
       </c>
-      <c r="J2">
+      <c r="J2" t="n">
         <v>185.3</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="1">
+    <row r="3">
+      <c r="A3" s="1" t="n">
         <v>45901</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="1" t="n">
         <v>45907</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>180.4</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>193.3</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>185.7</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>186.8</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>179.7</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="n">
         <v>179.9</v>
       </c>
-      <c r="I3">
+      <c r="I3" t="n">
         <v>188.5</v>
       </c>
-      <c r="J3">
+      <c r="J3" t="n">
         <v>185.7</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="1">
+    <row r="4">
+      <c r="A4" s="1" t="n">
         <v>45901</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="1" t="n">
         <v>45914</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>181</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>193.2</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>186.3</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>187.2</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>179.7</v>
       </c>
-      <c r="H4">
+      <c r="H4" t="n">
         <v>179.9</v>
       </c>
-      <c r="I4">
+      <c r="I4" t="n">
         <v>189.1</v>
       </c>
-      <c r="J4">
+      <c r="J4" t="n">
         <v>184.8</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="1">
+    <row r="5">
+      <c r="A5" s="1" t="n">
         <v>45901</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="1" t="n">
         <v>45921</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>181.1</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>193.1</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>186.6</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>187.4</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>179.1</v>
       </c>
-      <c r="H5">
+      <c r="H5" t="n">
         <v>179.8</v>
       </c>
-      <c r="I5">
+      <c r="I5" t="n">
         <v>189.2</v>
       </c>
-      <c r="J5">
+      <c r="J5" t="n">
         <v>184.7</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="1">
+    <row r="6">
+      <c r="A6" s="1" t="n">
         <v>45901</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="1" t="n">
         <v>45928</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>180.6</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>193.1</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>187.2</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>186.1</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>180.5</v>
       </c>
-      <c r="H6">
+      <c r="H6" t="n">
         <v>179.9</v>
       </c>
-      <c r="I6">
+      <c r="I6" t="n">
         <v>189.4</v>
       </c>
-      <c r="J6">
+      <c r="J6" t="n">
         <v>184.9</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="1">
+    <row r="7">
+      <c r="A7" s="1" t="n">
         <v>45931</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="1" t="n">
         <v>45935</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>180.6</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>193.4</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>186.4</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>185.7</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>180.1</v>
       </c>
-      <c r="H7">
+      <c r="H7" t="n">
         <v>179.9</v>
       </c>
-      <c r="I7">
+      <c r="I7" t="n">
         <v>189.6</v>
       </c>
-      <c r="J7">
+      <c r="J7" t="n">
         <v>185.6</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="1">
+    <row r="8">
+      <c r="A8" s="1" t="n">
         <v>45931</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="1" t="n">
         <v>45942</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>180.6</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>193.2</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>187.5</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>185.6</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>179.8</v>
       </c>
-      <c r="H8">
+      <c r="H8" t="n">
         <v>179.3</v>
       </c>
-      <c r="I8">
+      <c r="I8" t="n">
         <v>189.5</v>
       </c>
-      <c r="J8">
+      <c r="J8" t="n">
         <v>185.7</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="1">
+    <row r="9">
+      <c r="A9" s="1" t="n">
         <v>45931</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="1" t="n">
         <v>45949</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>180</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>193.1</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>185.4</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>185.1</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>179.3</v>
       </c>
-      <c r="H9">
+      <c r="H9" t="n">
         <v>178.7</v>
       </c>
-      <c r="I9">
+      <c r="I9" t="n">
         <v>189.1</v>
       </c>
-      <c r="J9">
+      <c r="J9" t="n">
         <v>185</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="1">
+    <row r="10">
+      <c r="A10" s="1" t="n">
         <v>45931</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="1" t="n">
         <v>45956</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>179.8</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>193.1</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>185.1</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>185</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>180.2</v>
       </c>
-      <c r="H10">
+      <c r="H10" t="n">
         <v>178.4</v>
       </c>
-      <c r="I10">
+      <c r="I10" t="n">
         <v>188.9</v>
       </c>
-      <c r="J10">
+      <c r="J10" t="n">
         <v>184.5</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="1">
+    <row r="11">
+      <c r="A11" s="1" t="n">
         <v>45962</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="1" t="n">
         <v>45963</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>180.5</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>193.2</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>186.5</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>187.2</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>180.7</v>
       </c>
-      <c r="H11">
+      <c r="H11" t="n">
         <v>179.9</v>
       </c>
-      <c r="I11">
+      <c r="I11" t="n">
         <v>188.5</v>
       </c>
-      <c r="J11">
+      <c r="J11" t="n">
         <v>185.8</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="1">
+    <row r="12">
+      <c r="A12" s="1" t="n">
         <v>45962</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="1" t="n">
         <v>45970</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="n">
         <v>181.7</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>193.4</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>187</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>188.3</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="n">
         <v>181.6</v>
       </c>
-      <c r="H12">
+      <c r="H12" t="n">
         <v>181.9</v>
       </c>
-      <c r="I12">
+      <c r="I12" t="n">
         <v>188.6</v>
       </c>
-      <c r="J12">
+      <c r="J12" t="n">
         <v>187.2</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="1">
+    <row r="13">
+      <c r="A13" s="1" t="n">
         <v>45962</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="1" t="n">
         <v>45977</v>
       </c>
-      <c r="C13">
+      <c r="C13" t="n">
         <v>185.3</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>195.7</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>190.5</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>190.9</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>184.3</v>
       </c>
-      <c r="H13">
+      <c r="H13" t="n">
         <v>184.6</v>
       </c>
-      <c r="I13">
+      <c r="I13" t="n">
         <v>189.7</v>
       </c>
-      <c r="J13">
+      <c r="J13" t="n">
         <v>188.5</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="1">
+    <row r="14">
+      <c r="A14" s="1" t="n">
         <v>45962</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="1" t="n">
         <v>45984</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="n">
         <v>188.5</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>199.2</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>193.2</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>193.2</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>188.4</v>
       </c>
-      <c r="H14">
+      <c r="H14" t="n">
         <v>187</v>
       </c>
-      <c r="I14">
+      <c r="I14" t="n">
         <v>191.5</v>
       </c>
-      <c r="J14">
+      <c r="J14" t="n">
         <v>191.3</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
-      <c r="A15" s="1">
+    <row r="15">
+      <c r="A15" s="1" t="n">
         <v>45962</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="1" t="n">
         <v>45991</v>
       </c>
-      <c r="C15">
+      <c r="C15" t="n">
         <v>189.2</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>201.8</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>194.1</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>194.9</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>189.8</v>
       </c>
-      <c r="H15">
+      <c r="H15" t="n">
         <v>188</v>
       </c>
-      <c r="I15">
+      <c r="I15" t="n">
         <v>192.4</v>
       </c>
-      <c r="J15">
+      <c r="J15" t="n">
         <v>193.9</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
-      <c r="A16" s="1">
+    <row r="16">
+      <c r="A16" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="1" t="n">
         <v>45998</v>
       </c>
-      <c r="C16">
+      <c r="C16" t="n">
         <v>188.6</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>202.4</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>194</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="n">
         <v>194.7</v>
       </c>
-      <c r="G16">
+      <c r="G16" t="n">
         <v>188.1</v>
       </c>
-      <c r="H16">
+      <c r="H16" t="n">
         <v>187</v>
       </c>
-      <c r="I16">
+      <c r="I16" t="n">
         <v>191.4</v>
       </c>
-      <c r="J16">
+      <c r="J16" t="n">
         <v>194.9</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
-      <c r="A17" s="1">
+    <row r="17">
+      <c r="A17" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="1" t="n">
         <v>46005</v>
       </c>
-      <c r="C17">
+      <c r="C17" t="n">
         <v>187.8</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="n">
         <v>202.2</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="n">
         <v>193.6</v>
       </c>
-      <c r="F17">
+      <c r="F17" t="n">
         <v>193.8</v>
       </c>
-      <c r="G17">
+      <c r="G17" t="n">
         <v>186.1</v>
       </c>
-      <c r="H17">
+      <c r="H17" t="n">
         <v>185.6</v>
       </c>
-      <c r="I17">
+      <c r="I17" t="n">
         <v>191</v>
       </c>
-      <c r="J17">
+      <c r="J17" t="n">
         <v>194.5</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
-      <c r="A18" s="1">
+    <row r="18">
+      <c r="A18" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="1" t="n">
         <v>46012</v>
       </c>
-      <c r="C18">
+      <c r="C18" t="n">
         <v>186.8</v>
       </c>
-      <c r="D18">
+      <c r="D18" t="n">
         <v>201.3</v>
       </c>
-      <c r="E18">
+      <c r="E18" t="n">
         <v>192.1</v>
       </c>
-      <c r="F18">
+      <c r="F18" t="n">
         <v>191.5</v>
       </c>
-      <c r="G18">
+      <c r="G18" t="n">
         <v>183.3</v>
       </c>
-      <c r="H18">
+      <c r="H18" t="n">
         <v>183.9</v>
       </c>
-      <c r="I18">
+      <c r="I18" t="n">
         <v>189.2</v>
       </c>
-      <c r="J18">
+      <c r="J18" t="n">
         <v>193</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
-      <c r="A19" s="1">
+    <row r="19">
+      <c r="A19" s="1" t="n">
         <v>45992</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="1" t="n">
         <v>46019</v>
       </c>
-      <c r="C19">
+      <c r="C19" t="n">
         <v>184.5</v>
       </c>
-      <c r="D19">
+      <c r="D19" t="n">
         <v>200.4</v>
       </c>
-      <c r="E19">
+      <c r="E19" t="n">
         <v>189.5</v>
       </c>
-      <c r="F19">
+      <c r="F19" t="n">
         <v>188.5</v>
       </c>
-      <c r="G19">
+      <c r="G19" t="n">
         <v>181.4</v>
       </c>
-      <c r="H19">
+      <c r="H19" t="n">
         <v>182.2</v>
       </c>
-      <c r="I19">
+      <c r="I19" t="n">
         <v>188</v>
       </c>
-      <c r="J19">
+      <c r="J19" t="n">
         <v>191.4</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
-      <c r="A20" s="1">
+    <row r="20">
+      <c r="A20" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="1" t="n">
         <v>46026</v>
       </c>
-      <c r="C20">
+      <c r="C20" t="n">
         <v>182</v>
       </c>
-      <c r="D20">
+      <c r="D20" t="n">
         <v>200.4</v>
       </c>
-      <c r="E20">
+      <c r="E20" t="n">
         <v>188.3</v>
       </c>
-      <c r="F20">
+      <c r="F20" t="n">
         <v>187</v>
       </c>
-      <c r="G20">
+      <c r="G20" t="n">
         <v>180.6</v>
       </c>
-      <c r="H20">
+      <c r="H20" t="n">
         <v>181.4</v>
       </c>
-      <c r="I20">
+      <c r="I20" t="n">
         <v>187.5</v>
       </c>
-      <c r="J20">
+      <c r="J20" t="n">
         <v>190</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
-      <c r="A21" s="1">
+    <row r="21">
+      <c r="A21" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="1" t="n">
         <v>46033</v>
       </c>
-      <c r="C21">
+      <c r="C21" t="n">
         <v>178.7</v>
       </c>
-      <c r="D21">
+      <c r="D21" t="n">
         <v>198.2</v>
       </c>
-      <c r="E21">
+      <c r="E21" t="n">
         <v>186.5</v>
       </c>
-      <c r="F21">
+      <c r="F21" t="n">
         <v>185.7</v>
       </c>
-      <c r="G21">
+      <c r="G21" t="n">
         <v>178.1</v>
       </c>
-      <c r="H21">
+      <c r="H21" t="n">
         <v>179.4</v>
       </c>
-      <c r="I21">
+      <c r="I21" t="n">
         <v>186.3</v>
       </c>
-      <c r="J21">
+      <c r="J21" t="n">
         <v>188.5</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
-      <c r="A22" s="1">
+    <row r="22">
+      <c r="A22" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="1" t="n">
         <v>46040</v>
       </c>
-      <c r="C22">
+      <c r="C22" t="n">
         <v>176.1</v>
       </c>
-      <c r="D22">
+      <c r="D22" t="n">
         <v>196.1</v>
       </c>
-      <c r="E22">
+      <c r="E22" t="n">
         <v>185.6</v>
       </c>
-      <c r="F22">
+      <c r="F22" t="n">
         <v>184.4</v>
       </c>
-      <c r="G22">
+      <c r="G22" t="n">
         <v>176.8</v>
       </c>
-      <c r="H22">
+      <c r="H22" t="n">
         <v>178.1</v>
       </c>
-      <c r="I22">
+      <c r="I22" t="n">
         <v>186.1</v>
       </c>
-      <c r="J22">
+      <c r="J22" t="n">
         <v>187.4</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
-      <c r="A23" s="1">
+    <row r="23">
+      <c r="A23" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="1" t="n">
         <v>46047</v>
       </c>
-      <c r="C23">
+      <c r="C23" t="n">
         <v>175.1</v>
       </c>
-      <c r="D23">
+      <c r="D23" t="n">
         <v>195.8</v>
       </c>
-      <c r="E23">
+      <c r="E23" t="n">
         <v>184.1</v>
       </c>
-      <c r="F23">
+      <c r="F23" t="n">
         <v>183</v>
       </c>
-      <c r="G23">
+      <c r="G23" t="n">
         <v>176.3</v>
       </c>
-      <c r="H23">
+      <c r="H23" t="n">
         <v>176.8</v>
       </c>
-      <c r="I23">
+      <c r="I23" t="n">
         <v>185.5</v>
       </c>
-      <c r="J23">
+      <c r="J23" t="n">
         <v>186.1</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
-      <c r="A24" s="1">
+    <row r="24">
+      <c r="A24" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="C24">
+      <c r="C24" t="n">
         <v>174.4</v>
       </c>
-      <c r="D24">
+      <c r="D24" t="n">
         <v>194.4</v>
       </c>
-      <c r="E24">
+      <c r="E24" t="n">
         <v>182.9</v>
       </c>
-      <c r="F24">
+      <c r="F24" t="n">
         <v>181.9</v>
       </c>
-      <c r="G24">
+      <c r="G24" t="n">
         <v>175.3</v>
       </c>
-      <c r="H24">
+      <c r="H24" t="n">
         <v>176.2</v>
       </c>
-      <c r="I24">
+      <c r="I24" t="n">
         <v>184.1</v>
       </c>
-      <c r="J24">
+      <c r="J24" t="n">
         <v>185.6</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
-      <c r="A25" s="1">
+    <row r="25">
+      <c r="A25" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="1" t="n">
         <v>46061</v>
       </c>
-      <c r="C25">
+      <c r="C25" t="n">
         <v>173.7</v>
       </c>
-      <c r="D25">
+      <c r="D25" t="n">
         <v>189.7</v>
       </c>
-      <c r="E25">
+      <c r="E25" t="n">
         <v>181.6</v>
       </c>
-      <c r="F25">
+      <c r="F25" t="n">
         <v>181</v>
       </c>
-      <c r="G25">
+      <c r="G25" t="n">
         <v>174.9</v>
       </c>
-      <c r="H25">
+      <c r="H25" t="n">
         <v>176.2</v>
       </c>
-      <c r="I25">
+      <c r="I25" t="n">
         <v>183.1</v>
       </c>
-      <c r="J25">
+      <c r="J25" t="n">
         <v>185.3</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
-      <c r="A26" s="1">
+    <row r="26">
+      <c r="A26" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="C26">
+      <c r="C26" t="n">
         <v>173.9</v>
       </c>
-      <c r="D26">
+      <c r="D26" t="n">
         <v>186.9</v>
       </c>
-      <c r="E26">
+      <c r="E26" t="n">
         <v>179.8</v>
       </c>
-      <c r="F26">
+      <c r="F26" t="n">
         <v>181.1</v>
       </c>
-      <c r="G26">
+      <c r="G26" t="n">
         <v>175.1</v>
       </c>
-      <c r="H26">
+      <c r="H26" t="n">
         <v>176.1</v>
       </c>
-      <c r="I26">
+      <c r="I26" t="n">
         <v>182.6</v>
       </c>
-      <c r="J26">
+      <c r="J26" t="n">
         <v>184.1</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
-      <c r="A27" s="1">
+    <row r="27">
+      <c r="A27" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="1" t="n">
         <v>46075</v>
       </c>
-      <c r="C27">
+      <c r="C27" t="n">
         <v>174.1</v>
       </c>
-      <c r="D27">
+      <c r="D27" t="n">
         <v>186.9</v>
       </c>
-      <c r="E27">
+      <c r="E27" t="n">
         <v>179.2</v>
       </c>
-      <c r="F27">
+      <c r="F27" t="n">
         <v>180.5</v>
       </c>
-      <c r="G27">
+      <c r="G27" t="n">
         <v>175</v>
       </c>
-      <c r="H27">
+      <c r="H27" t="n">
         <v>175.8</v>
       </c>
-      <c r="I27">
+      <c r="I27" t="n">
         <v>182.5</v>
       </c>
-      <c r="J27">
+      <c r="J27" t="n">
         <v>182.1</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
-      <c r="A28" s="1">
+    <row r="28">
+      <c r="A28" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="C28">
+      <c r="C28" t="n">
         <v>175.4</v>
       </c>
-      <c r="D28">
+      <c r="D28" t="n">
         <v>187</v>
       </c>
-      <c r="E28">
+      <c r="E28" t="n">
         <v>180.3</v>
       </c>
-      <c r="F28">
+      <c r="F28" t="n">
         <v>181.9</v>
       </c>
-      <c r="G28">
+      <c r="G28" t="n">
         <v>175.6</v>
       </c>
-      <c r="H28">
+      <c r="H28" t="n">
         <v>176.7</v>
       </c>
-      <c r="I28">
+      <c r="I28" t="n">
         <v>183.6</v>
       </c>
-      <c r="J28">
+      <c r="J28" t="n">
         <v>183.2</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
-      <c r="A29" s="1">
+    <row r="29">
+      <c r="A29" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="1" t="n">
         <v>46089</v>
       </c>
-      <c r="C29">
+      <c r="C29" t="n">
         <v>197.4</v>
       </c>
-      <c r="D29">
+      <c r="D29" t="n">
         <v>198.9</v>
       </c>
-      <c r="E29">
+      <c r="E29" t="n">
         <v>195.3</v>
       </c>
-      <c r="F29">
+      <c r="F29" t="n">
         <v>199.4</v>
       </c>
-      <c r="G29">
+      <c r="G29" t="n">
         <v>192.1</v>
       </c>
-      <c r="H29">
+      <c r="H29" t="n">
         <v>190.5</v>
       </c>
-      <c r="I29">
+      <c r="I29" t="n">
         <v>199.5</v>
       </c>
-      <c r="J29">
+      <c r="J29" t="n">
         <v>198.6</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
-      <c r="A30" s="1">
+    <row r="30">
+      <c r="A30" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="1" t="n">
         <v>46096</v>
       </c>
-      <c r="C30">
+      <c r="C30" t="n">
         <v>247.2</v>
       </c>
-      <c r="D30">
+      <c r="D30" t="n">
         <v>246.4</v>
       </c>
-      <c r="E30">
+      <c r="E30" t="n">
         <v>244.1</v>
       </c>
-      <c r="F30">
+      <c r="F30" t="n">
         <v>245.9</v>
       </c>
-      <c r="G30">
+      <c r="G30" t="n">
         <v>245.1</v>
       </c>
-      <c r="H30">
+      <c r="H30" t="n">
         <v>244.3</v>
       </c>
-      <c r="I30">
+      <c r="I30" t="n">
         <v>247</v>
       </c>
-      <c r="J30">
+      <c r="J30" t="n">
         <v>245.3</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
-      <c r="A31" s="1">
+    <row r="31">
+      <c r="A31" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="1" t="n">
         <v>46103</v>
       </c>
-      <c r="C31">
+      <c r="C31" t="n">
         <v>282.1</v>
       </c>
-      <c r="D31">
+      <c r="D31" t="n">
         <v>282.5</v>
       </c>
-      <c r="E31">
+      <c r="E31" t="n">
         <v>282.1</v>
       </c>
-      <c r="F31">
+      <c r="F31" t="n">
         <v>281.7</v>
       </c>
-      <c r="G31">
+      <c r="G31" t="n">
         <v>280.6</v>
       </c>
-      <c r="H31">
+      <c r="H31" t="n">
         <v>279.2</v>
       </c>
-      <c r="I31">
+      <c r="I31" t="n">
         <v>281.6</v>
       </c>
-      <c r="J31">
+      <c r="J31" t="n">
         <v>279.9</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
-      <c r="A32" s="1">
+    <row r="32">
+      <c r="A32" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="1" t="n">
         <v>46110</v>
       </c>
-      <c r="C32">
+      <c r="C32" t="n">
         <v>309.1</v>
       </c>
-      <c r="D32">
+      <c r="D32" t="n">
         <v>309.1</v>
       </c>
-      <c r="E32">
+      <c r="E32" t="n">
         <v>309</v>
       </c>
-      <c r="F32">
+      <c r="F32" t="n">
         <v>310.3</v>
       </c>
-      <c r="G32">
+      <c r="G32" t="n">
         <v>308.9</v>
       </c>
-      <c r="H32">
+      <c r="H32" t="n">
         <v>305.4</v>
       </c>
-      <c r="I32">
+      <c r="I32" t="n">
         <v>308</v>
       </c>
-      <c r="J32">
+      <c r="J32" t="n">
         <v>307.8</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
-      <c r="A33" s="1">
+    <row r="33">
+      <c r="A33" s="1" t="n">
         <v>46113</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="1" t="n">
         <v>46117</v>
       </c>
-      <c r="C33">
+      <c r="C33" t="n">
         <v>310.6</v>
       </c>
-      <c r="D33">
+      <c r="D33" t="n">
         <v>308.5</v>
       </c>
-      <c r="E33">
+      <c r="E33" t="n">
         <v>311.8</v>
       </c>
-      <c r="F33">
+      <c r="F33" t="n">
         <v>310.2</v>
       </c>
-      <c r="G33">
+      <c r="G33" t="n">
         <v>308.8</v>
       </c>
-      <c r="H33">
+      <c r="H33" t="n">
         <v>309</v>
       </c>
-      <c r="I33">
+      <c r="I33" t="n">
         <v>309.5</v>
       </c>
-      <c r="J33">
+      <c r="J33" t="n">
         <v>306.1</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
-      <c r="A34" s="1">
+    <row r="34">
+      <c r="A34" s="1" t="n">
         <v>46113</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="1" t="n">
         <v>46124</v>
       </c>
-      <c r="C34">
+      <c r="C34" t="n">
         <v>316</v>
       </c>
-      <c r="D34">
+      <c r="D34" t="n">
         <v>317.7</v>
       </c>
-      <c r="E34">
+      <c r="E34" t="n">
         <v>317.9</v>
       </c>
-      <c r="F34">
+      <c r="F34" t="n">
         <v>318.3</v>
       </c>
-      <c r="G34">
+      <c r="G34" t="n">
         <v>318.2</v>
       </c>
-      <c r="H34">
+      <c r="H34" t="n">
         <v>315.4</v>
       </c>
-      <c r="I34">
+      <c r="I34" t="n">
         <v>319.3</v>
       </c>
-      <c r="J34">
+      <c r="J34" t="n">
         <v>316.6</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
-      <c r="A35" s="1">
+    <row r="35">
+      <c r="A35" s="1" t="n">
         <v>46113</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="1" t="n">
         <v>46131</v>
       </c>
-      <c r="C35">
+      <c r="C35" t="n">
         <v>304.1</v>
       </c>
-      <c r="D35">
+      <c r="D35" t="n">
         <v>302.6</v>
       </c>
-      <c r="E35">
+      <c r="E35" t="n">
         <v>306.1</v>
       </c>
-      <c r="F35">
+      <c r="F35" t="n">
         <v>308.7</v>
       </c>
-      <c r="G35">
+      <c r="G35" t="n">
         <v>304.3</v>
       </c>
-      <c r="H35">
+      <c r="H35" t="n">
         <v>301.3</v>
       </c>
-      <c r="I35">
+      <c r="I35" t="n">
         <v>305.6</v>
       </c>
-      <c r="J35">
+      <c r="J35" t="n">
         <v>302.1</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
-      <c r="A36" s="1">
+    <row r="36">
+      <c r="A36" s="1" t="n">
         <v>46113</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="1" t="n">
         <v>46138</v>
       </c>
-      <c r="C36">
+      <c r="C36" t="n">
         <v>268.5</v>
       </c>
-      <c r="D36">
+      <c r="D36" t="n">
         <v>277</v>
       </c>
-      <c r="E36">
+      <c r="E36" t="n">
         <v>274.1</v>
       </c>
-      <c r="F36">
+      <c r="F36" t="n">
         <v>271.3</v>
       </c>
-      <c r="G36">
+      <c r="G36" t="n">
         <v>266.8</v>
       </c>
-      <c r="H36">
+      <c r="H36" t="n">
         <v>263.3</v>
       </c>
-      <c r="I36">
+      <c r="I36" t="n">
         <v>274.6</v>
       </c>
-      <c r="J36">
+      <c r="J36" t="n">
         <v>266.8</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
-      <c r="A37" s="1">
+    <row r="37">
+      <c r="A37" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="B37" s="1">
+      <c r="B37" s="1" t="n">
         <v>46145</v>
       </c>
-      <c r="C37">
+      <c r="C37" t="n">
         <v>246.9</v>
       </c>
-      <c r="D37">
+      <c r="D37" t="n">
         <v>268.5</v>
       </c>
-      <c r="E37">
+      <c r="E37" t="n">
         <v>253</v>
       </c>
-      <c r="F37">
+      <c r="F37" t="n">
         <v>250.6</v>
       </c>
-      <c r="G37">
+      <c r="G37" t="n">
         <v>243.9</v>
       </c>
-      <c r="H37">
+      <c r="H37" t="n">
         <v>243.1</v>
       </c>
-      <c r="I37">
+      <c r="I37" t="n">
         <v>253.4</v>
       </c>
-      <c r="J37">
+      <c r="J37" t="n">
         <v>251.5</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
-      <c r="A38" s="1">
+    <row r="38">
+      <c r="A38" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="1" t="n">
         <v>46152</v>
       </c>
-      <c r="C38">
+      <c r="C38" t="n">
         <v>239.9</v>
       </c>
-      <c r="D38">
+      <c r="D38" t="n">
         <v>265.3</v>
       </c>
-      <c r="E38">
+      <c r="E38" t="n">
         <v>247.1</v>
       </c>
-      <c r="F38">
+      <c r="F38" t="n">
         <v>243.9</v>
       </c>
-      <c r="G38">
+      <c r="G38" t="n">
         <v>238.9</v>
       </c>
-      <c r="H38">
+      <c r="H38" t="n">
         <v>236.2</v>
       </c>
-      <c r="I38">
+      <c r="I38" t="n">
         <v>247.7</v>
       </c>
-      <c r="J38">
+      <c r="J38" t="n">
         <v>247.2</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
-      <c r="A39" s="1">
+    <row r="39">
+      <c r="A39" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="1" t="n">
         <v>46159</v>
       </c>
-      <c r="C39">
+      <c r="C39" t="n">
         <v>231</v>
       </c>
-      <c r="D39">
+      <c r="D39" t="n">
         <v>260.1</v>
       </c>
-      <c r="E39">
+      <c r="E39" t="n">
         <v>239.1</v>
       </c>
-      <c r="F39">
+      <c r="F39" t="n">
         <v>233.8</v>
       </c>
-      <c r="G39">
+      <c r="G39" t="n">
         <v>229.9</v>
       </c>
-      <c r="H39">
+      <c r="H39" t="n">
         <v>222.9</v>
       </c>
-      <c r="I39">
+      <c r="I39" t="n">
         <v>240.8</v>
       </c>
-      <c r="J39">
+      <c r="J39" t="n">
         <v>236.2</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
-      <c r="A40" s="1">
+    <row r="40">
+      <c r="A40" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="1" t="n">
         <v>46166</v>
       </c>
-      <c r="C40">
+      <c r="C40" t="n">
         <v>225.8</v>
       </c>
-      <c r="D40">
+      <c r="D40" t="n">
         <v>258.3</v>
       </c>
-      <c r="E40">
+      <c r="E40" t="n">
         <v>232.7</v>
       </c>
-      <c r="F40">
+      <c r="F40" t="n">
         <v>228.5</v>
       </c>
-      <c r="G40">
+      <c r="G40" t="n">
         <v>224.5</v>
       </c>
-      <c r="H40">
+      <c r="H40" t="n">
         <v>217.3</v>
       </c>
-      <c r="I40">
+      <c r="I40" t="n">
         <v>236.2</v>
       </c>
-      <c r="J40">
+      <c r="J40" t="n">
         <v>230.4</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
-      <c r="A41" s="1">
+    <row r="41">
+      <c r="A41" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="1" t="n">
         <v>46173</v>
       </c>
-      <c r="C41">
+      <c r="C41" t="n">
         <v>219.3</v>
       </c>
-      <c r="D41">
+      <c r="D41" t="n">
         <v>248.1</v>
       </c>
-      <c r="E41">
+      <c r="E41" t="n">
         <v>225.5</v>
       </c>
-      <c r="F41">
+      <c r="F41" t="n">
         <v>223.4</v>
       </c>
-      <c r="G41">
+      <c r="G41" t="n">
         <v>217.5</v>
       </c>
-      <c r="H41">
+      <c r="H41" t="n">
         <v>211.6</v>
       </c>
-      <c r="I41">
+      <c r="I41" t="n">
         <v>229</v>
       </c>
-      <c r="J41">
+      <c r="J41" t="n">
         <v>226.5</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
-      <c r="A42" s="1">
+    <row r="42">
+      <c r="A42" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="1" t="n">
         <v>46180</v>
       </c>
-      <c r="C42">
+      <c r="C42" t="n">
         <v>204.7</v>
       </c>
-      <c r="D42">
+      <c r="D42" t="n">
         <v>221.8</v>
       </c>
-      <c r="E42">
+      <c r="E42" t="n">
         <v>213.3</v>
       </c>
-      <c r="F42">
+      <c r="F42" t="n">
         <v>212.4</v>
       </c>
-      <c r="G42">
+      <c r="G42" t="n">
         <v>206</v>
       </c>
-      <c r="H42">
+      <c r="H42" t="n">
         <v>201</v>
       </c>
-      <c r="I42">
+      <c r="I42" t="n">
         <v>210.3</v>
       </c>
-      <c r="J42">
+      <c r="J42" t="n">
         <v>219.4</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
-      <c r="A43" s="1">
+    <row r="43">
+      <c r="A43" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="1" t="n">
         <v>46187</v>
       </c>
-      <c r="C43">
+      <c r="C43" t="n">
         <v>197.2</v>
       </c>
-      <c r="D43">
+      <c r="D43" t="n">
         <v>214.4</v>
       </c>
-      <c r="E43">
+      <c r="E43" t="n">
         <v>206.3</v>
       </c>
-      <c r="F43">
+      <c r="F43" t="n">
         <v>205.1</v>
       </c>
-      <c r="G43">
+      <c r="G43" t="n">
         <v>201.3</v>
       </c>
-      <c r="H43">
+      <c r="H43" t="n">
         <v>194.7</v>
       </c>
-      <c r="I43">
+      <c r="I43" t="n">
         <v>199.2</v>
       </c>
-      <c r="J43">
+      <c r="J43" t="n">
         <v>215</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
-      <c r="A44" s="1">
+    <row r="44">
+      <c r="A44" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="1" t="n">
         <v>46194</v>
       </c>
-      <c r="C44">
+      <c r="C44" t="n">
         <v>189.3</v>
       </c>
-      <c r="D44">
+      <c r="D44" t="n">
         <v>203</v>
       </c>
-      <c r="E44">
+      <c r="E44" t="n">
         <v>195.4</v>
       </c>
-      <c r="F44">
+      <c r="F44" t="n">
         <v>195.9</v>
       </c>
-      <c r="G44">
+      <c r="G44" t="n">
         <v>194</v>
       </c>
-      <c r="H44">
+      <c r="H44" t="n">
         <v>188</v>
       </c>
-      <c r="I44">
+      <c r="I44" t="n">
         <v>192.5</v>
       </c>
-      <c r="J44">
+      <c r="J44" t="n">
         <v>205.6</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
-      <c r="A45" s="1">
+    <row r="45">
+      <c r="A45" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="1" t="n">
         <v>46201</v>
       </c>
-      <c r="C45">
+      <c r="C45" t="n">
         <v>177.3</v>
       </c>
-      <c r="D45">
+      <c r="D45" t="n">
         <v>196.2</v>
       </c>
-      <c r="E45">
+      <c r="E45" t="n">
         <v>180.9</v>
       </c>
-      <c r="F45">
+      <c r="F45" t="n">
         <v>181.7</v>
       </c>
-      <c r="G45">
+      <c r="G45" t="n">
         <v>180.3</v>
       </c>
-      <c r="H45">
+      <c r="H45" t="n">
         <v>174.3</v>
       </c>
-      <c r="I45">
+      <c r="I45" t="n">
         <v>182</v>
       </c>
-      <c r="J45">
+      <c r="J45" t="n">
         <v>192.6</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
-      <c r="A46" s="1">
+    <row r="46">
+      <c r="A46" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="1" t="n">
         <v>46208</v>
       </c>
-      <c r="C46">
+      <c r="C46" t="n">
         <v>180.5</v>
       </c>
-      <c r="D46">
+      <c r="D46" t="n">
         <v>193.4</v>
       </c>
-      <c r="E46">
+      <c r="E46" t="n">
         <v>181.8</v>
       </c>
-      <c r="F46">
+      <c r="F46" t="n">
         <v>182.9</v>
       </c>
-      <c r="G46">
+      <c r="G46" t="n">
         <v>181.4</v>
       </c>
-      <c r="H46">
+      <c r="H46" t="n">
         <v>177.7</v>
       </c>
-      <c r="I46">
+      <c r="I46" t="n">
         <v>182.5</v>
       </c>
-      <c r="J46">
+      <c r="J46" t="n">
         <v>195.9</v>
       </c>
     </row>
-    <row r="47" spans="1:10">
-      <c r="A47" s="1">
+    <row r="47">
+      <c r="A47" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="1" t="n">
         <v>46215</v>
       </c>
-      <c r="C47">
+      <c r="C47" t="n">
         <v>185.8</v>
       </c>
-      <c r="D47">
+      <c r="D47" t="n">
         <v>200.3</v>
       </c>
-      <c r="E47">
+      <c r="E47" t="n">
         <v>187.7</v>
       </c>
-      <c r="F47">
+      <c r="F47" t="n">
         <v>188.2</v>
       </c>
-      <c r="G47">
+      <c r="G47" t="n">
         <v>187.2</v>
       </c>
-      <c r="H47">
+      <c r="H47" t="n">
         <v>182.8</v>
       </c>
-      <c r="I47">
+      <c r="I47" t="n">
         <v>188.9</v>
       </c>
-      <c r="J47">
+      <c r="J47" t="n">
         <v>199.1</v>
       </c>
     </row>
-    <row r="48" spans="1:10">
-      <c r="A48" s="1">
+    <row r="48">
+      <c r="A48" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="1" t="n">
         <v>46222</v>
       </c>
-      <c r="C48">
+      <c r="C48" t="n">
         <v>197.7</v>
       </c>
-      <c r="D48">
+      <c r="D48" t="n">
         <v>201.3</v>
       </c>
-      <c r="E48">
+      <c r="E48" t="n">
         <v>199.2</v>
       </c>
-      <c r="F48">
+      <c r="F48" t="n">
         <v>200</v>
       </c>
-      <c r="G48">
+      <c r="G48" t="n">
         <v>196.3</v>
       </c>
-      <c r="H48">
+      <c r="H48" t="n">
         <v>193.4</v>
       </c>
-      <c r="I48">
+      <c r="I48" t="n">
         <v>200</v>
       </c>
-      <c r="J48">
+      <c r="J48" t="n">
         <v>204.2</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
-      <c r="A49" s="1">
+    <row r="49">
+      <c r="A49" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="B49" s="1">
+      <c r="B49" s="1" t="n">
         <v>46229</v>
       </c>
-      <c r="C49">
+      <c r="C49" t="n">
         <v>217.8</v>
       </c>
-      <c r="D49">
+      <c r="D49" t="n">
         <v>221.9</v>
       </c>
-      <c r="E49">
+      <c r="E49" t="n">
         <v>220.5</v>
       </c>
-      <c r="F49">
+      <c r="F49" t="n">
         <v>219.4</v>
       </c>
-      <c r="G49">
+      <c r="G49" t="n">
         <v>218.1</v>
       </c>
-      <c r="H49">
+      <c r="H49" t="n">
         <v>212.4</v>
       </c>
-      <c r="I49">
+      <c r="I49" t="n">
         <v>221.3</v>
       </c>
-      <c r="J49">
+      <c r="J49" t="n">
         <v>221.4</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
-      <c r="A50" s="1">
+    <row r="50">
+      <c r="A50" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="1" t="n">
         <v>46236</v>
       </c>
-      <c r="C50">
+      <c r="C50" t="n">
         <v>233.2</v>
       </c>
-      <c r="D50">
+      <c r="D50" t="n">
         <v>239.7</v>
       </c>
-      <c r="E50">
+      <c r="E50" t="n">
         <v>237</v>
       </c>
-      <c r="F50">
+      <c r="F50" t="n">
         <v>234.6</v>
       </c>
-      <c r="G50">
+      <c r="G50" t="n">
         <v>234</v>
       </c>
-      <c r="H50">
+      <c r="H50" t="n">
         <v>227.1</v>
       </c>
-      <c r="I50">
+      <c r="I50" t="n">
         <v>239.5</v>
       </c>
-      <c r="J50">
+      <c r="J50" t="n">
         <v>237.6</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
-      <c r="A51" s="1">
+    <row r="51">
+      <c r="A51" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B51" s="1" t="n">
         <v>46243</v>
       </c>
-      <c r="C51">
+      <c r="C51" t="n">
         <v>244.4</v>
       </c>
-      <c r="D51">
+      <c r="D51" t="n">
         <v>253.9</v>
       </c>
-      <c r="E51">
+      <c r="E51" t="n">
         <v>250.6</v>
       </c>
-      <c r="F51">
+      <c r="F51" t="n">
         <v>247.7</v>
       </c>
-      <c r="G51">
+      <c r="G51" t="n">
         <v>247.3</v>
       </c>
-      <c r="H51">
+      <c r="H51" t="n">
         <v>241.4</v>
       </c>
-      <c r="I51">
+      <c r="I51" t="n">
         <v>253.1</v>
       </c>
-      <c r="J51">
+      <c r="J51" t="n">
         <v>251.9</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
-      <c r="A52" s="1">
+    <row r="52">
+      <c r="A52" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="B52" s="1">
+      <c r="B52" s="1" t="n">
         <v>46250</v>
       </c>
-      <c r="C52">
+      <c r="C52" t="n">
         <v>239.9</v>
       </c>
-      <c r="D52">
+      <c r="D52" t="n">
         <v>244.8</v>
       </c>
-      <c r="E52">
+      <c r="E52" t="n">
         <v>244.9</v>
       </c>
-      <c r="F52">
+      <c r="F52" t="n">
         <v>245</v>
       </c>
-      <c r="G52">
+      <c r="G52" t="n">
         <v>241.5</v>
       </c>
-      <c r="H52">
+      <c r="H52" t="n">
         <v>238.1</v>
       </c>
-      <c r="I52">
+      <c r="I52" t="n">
         <v>250</v>
       </c>
-      <c r="J52">
+      <c r="J52" t="n">
         <v>248.9</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
-      <c r="A53" s="1">
+    <row r="53">
+      <c r="A53" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="B53" s="1">
+      <c r="B53" s="1" t="n">
         <v>46257</v>
       </c>
-      <c r="C53">
+      <c r="C53" t="n">
         <v>242.9</v>
       </c>
-      <c r="D53">
+      <c r="D53" t="n">
         <v>251.7</v>
       </c>
-      <c r="E53">
+      <c r="E53" t="n">
         <v>248.5</v>
       </c>
-      <c r="F53">
+      <c r="F53" t="n">
         <v>247.9</v>
       </c>
-      <c r="G53">
+      <c r="G53" t="n">
         <v>244.9</v>
       </c>
-      <c r="H53">
+      <c r="H53" t="n">
         <v>242.2</v>
       </c>
-      <c r="I53">
+      <c r="I53" t="n">
         <v>251.9</v>
       </c>
-      <c r="J53">
+      <c r="J53" t="n">
         <v>251</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>